<commit_message>
Actualizacao dos graficos de sustentabilidade
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -691,6 +691,91 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>2026-06-24 10:17:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:50:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-06-29 17:20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-06-30 15:20:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-06-30 16:04:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-07-02 14:36:47</t>
         </is>
       </c>
     </row>
@@ -955,13 +1040,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50B5A53C-B107-4D06-88D6-01C8396D6F34}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BC51638-3A33-46CC-8F13-83B0CDEEACC4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B7506CC5-549B-4FCC-A76F-5D3979F5E547}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFA8390C-73DD-474C-B7C1-A4ACBE12ED4A}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{780CE8FE-5765-478F-B4A5-E8890DA3024F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{548CB65D-09E6-4745-8BC8-88A81D4D1C1A}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao das paginas e graficos
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -776,6 +776,23 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>2026-07-02 14:36:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-07-08 15:47:08</t>
         </is>
       </c>
     </row>
@@ -1040,13 +1057,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5BC51638-3A33-46CC-8F13-83B0CDEEACC4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CCE11D62-A66E-4216-8B1F-7E425D7B37BB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFA8390C-73DD-474C-B7C1-A4ACBE12ED4A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB66CD6E-08FC-4ED2-ADD1-EF4C8370899D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{548CB65D-09E6-4745-8BC8-88A81D4D1C1A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53DE486C-EA81-4751-A760-3D320FD0A965}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao e interpretacao dos dados baseline
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -813,274 +813,24 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-07-15 13:37:38</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
-    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
-    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66D0258C-A8E0-45EB-9991-83ACF908787C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8BC6793-A71E-467D-9434-1D5FB47493DC}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{002569A9-1667-4506-B803-9322248FAB24}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao dos dados analises financeira
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -830,7 +830,291 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:03:35</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="481cb719fb2f51215cc00c8d40533043">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="71df0815368817fe9627576b1e062219" ns2:_="" ns3:_="">
+    <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <xsd:import namespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="20d57abc-823c-4051-a81a-1a0a01a8f39e" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="16" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="19" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="edc6e55a-975c-4e83-894d-449406ca2714" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="21" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="22" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="54c5ab46-7543-4aba-b0fa-79d6a199bef5" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="20" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{21a739d7-e82a-41d6-a891-a689fdcdcba6}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="54c5ab46-7543-4aba-b0fa-79d6a199bef5">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E79B6761-FBE3-4117-9AA0-A003C4360AA3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32DACE4A-8BF4-4C53-AF50-4374B1789790}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89D5D084-131E-4035-85E7-39D3A4D1BDB1}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacão dadosfinanceiros e paginas da Beira
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -946,6 +946,40 @@
       <c r="C35" t="inlineStr">
         <is>
           <t>2026-07-21 16:26:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-07-24 11:36:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-07-24 13:06:05</t>
         </is>
       </c>
     </row>
@@ -1210,13 +1244,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9E0C59-CAAB-4359-B1A1-E8B6900664A1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EA278026-4A8B-41B8-9098-0632D5457457}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2B1E1FA-0E66-4FB4-9F53-32F8A1290DA0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F665A24-04BC-43D8-A71A-86BF1F545C66}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FBDD0FAD-D0F0-4AB4-AF39-FEFB91E7708D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8838476-5D29-49B1-8C37-1BC5FA1A89CC}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao dos resultados dos exercicios
</commit_message>
<xml_diff>
--- a/log_acoes.xlsx
+++ b/log_acoes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1116,6 +1116,23 @@
       <c r="C45" t="inlineStr">
         <is>
           <t>2026-08-06 12:02:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Atualizou os dados</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-08-24 16:40:34</t>
         </is>
       </c>
     </row>
@@ -1380,13 +1397,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{238FD987-3A8D-4B76-AF1C-3176A19ADE75}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{926A8941-91AE-44B5-8AB9-0D1CACADD2AC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{781EFE65-A72E-4048-B161-FC246A909A18}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D574EB3C-68DF-4E12-B409-25724EE31568}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3B42184-1256-4D8E-9468-9A60FD7962D6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FF05007-6153-47EA-996E-9F71969C83DE}"/>
 </file>
</xml_diff>